<commit_message>
26.02.12 Added Alternate Test and Alternate District fields to the DRC MSU roster file. Also updated the data dictionary and changed the student test page to show the alternate school/district options for students in 10th (only taking the science assessment).
</commit_message>
<xml_diff>
--- a/Science MSU Data Dictionary.xlsx
+++ b/Science MSU Data Dictionary.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Repos\AKPSUG-Accom\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{177B5CFC-38F2-4B57-8890-61D7ABD4907C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{564A0955-848B-4076-B588-37C1C150EB33}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="560" yWindow="5960" windowWidth="23430" windowHeight="12560" xr2:uid="{738CAF26-924C-4743-B4B5-7BBD7404522E}"/>
+    <workbookView xWindow="-35630" yWindow="290" windowWidth="33070" windowHeight="19990" xr2:uid="{738CAF26-924C-4743-B4B5-7BBD7404522E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="75">
   <si>
     <t>District Code</t>
   </si>
@@ -272,6 +272,18 @@
   </si>
   <si>
     <t>State Defined student race code (Replaces fields 13-17)</t>
+  </si>
+  <si>
+    <t>Alternate District</t>
+  </si>
+  <si>
+    <t>Alternate School</t>
+  </si>
+  <si>
+    <t>Alternate Test School ID, if set on the student page.</t>
+  </si>
+  <si>
+    <t>Alternate Test District ID, if set on the student page.</t>
   </si>
 </sst>
 </file>
@@ -450,8 +462,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7950601A-D55A-408B-AACA-62334041F2E4}" name="Table1" displayName="Table1" ref="A1:D29" totalsRowShown="0">
-  <autoFilter ref="A1:D29" xr:uid="{CCE2467A-F933-40C7-99A1-3B246FB54958}">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{7950601A-D55A-408B-AACA-62334041F2E4}" name="Table1" displayName="Table1" ref="A1:D31" totalsRowShown="0">
+  <autoFilter ref="A1:D31" xr:uid="{CCE2467A-F933-40C7-99A1-3B246FB54958}">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -764,7 +776,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7511A7ED-2D6F-4294-AFFE-C363D701DA2B}">
-  <dimension ref="A1:D29"/>
+  <dimension ref="A1:D31"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="2.36328125" style="7" customWidth="1"/>
@@ -1163,6 +1175,34 @@
       </c>
       <c r="D29" s="3" t="s">
         <v>70</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A30" s="9">
+        <v>29</v>
+      </c>
+      <c r="B30" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A31" s="9">
+        <v>30</v>
+      </c>
+      <c r="B31" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>

</xml_diff>